<commit_message>
18/08/2026 changes in the storage code to have the good equations for the by_pass
</commit_message>
<xml_diff>
--- a/Storage/Profiles_For_Energy_Storage.xlsx
+++ b/Storage/Profiles_For_Energy_Storage.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://insalyonfrance-my.sharepoint.com/personal/sserranose_insa-lyon_fr/Documents/Bureau/Code/Panda_pipes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://insalyonfrance-my.sharepoint.com/personal/sserranose_insa-lyon_fr/Documents/Bureau/Code/Panda_pipes/Storage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="14_{AE8AFB5B-C24D-4FF3-A185-DE1B94EC8289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D7643F4-4010-4421-923D-86F7B1C77349}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="14_{AE8AFB5B-C24D-4FF3-A185-DE1B94EC8289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4C9B9D3-224C-4259-8659-133706A35945}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1470" windowWidth="29040" windowHeight="15720" xr2:uid="{CDA0643C-BAC3-467D-87B4-54BBFD1AB2F5}"/>
+    <workbookView xWindow="-23550" yWindow="4305" windowWidth="19200" windowHeight="9555" xr2:uid="{CDA0643C-BAC3-467D-87B4-54BBFD1AB2F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -452,9 +452,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17706927-21CD-4346-BB1B-EE8F8F2B9564}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="3" max="4" width="14" bestFit="1" customWidth="1"/>
     <col min="5" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -522,7 +523,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
-        <f t="shared" ref="A4:A12" si="0">B4/3600</f>
+        <f t="shared" ref="A4:A13" si="0">B4/3600</f>
         <v>2</v>
       </c>
       <c r="B4">
@@ -697,16 +698,37 @@
         <v>36000</v>
       </c>
       <c r="C12" s="1">
+        <v>75000</v>
+      </c>
+      <c r="D12" s="1">
+        <v>150000</v>
+      </c>
+      <c r="E12" s="1">
+        <v>150000</v>
+      </c>
+      <c r="F12" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>39600</v>
+      </c>
+      <c r="C13" s="1">
         <v>37500</v>
       </c>
-      <c r="D12" s="2">
-        <v>0</v>
-      </c>
-      <c r="E12" s="1">
-        <v>150000</v>
-      </c>
-      <c r="F12" s="3">
-        <v>0.1</v>
+      <c r="D13" s="2">
+        <v>0</v>
+      </c>
+      <c r="E13" s="1">
+        <v>150000</v>
+      </c>
+      <c r="F13" s="3">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>